<commit_message>
ingesta: snapshot 2026-07-17 18:11 UTC
</commit_message>
<xml_diff>
--- a/data_lake/acumulado_tempmax_mes/dt=2026-07-17/Temp-max-julio-26.xlsx
+++ b/data_lake/acumulado_tempmax_mes/dt=2026-07-17/Temp-max-julio-26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.187.8\Oficina\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{406E136C-DDF1-48F7-A97C-16127752DD4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFDA2798-C1DC-46BE-A721-D5052D7B68C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TMAX_PRINCIPALES_CIUDADES" sheetId="1" r:id="rId1"/>
@@ -1219,7 +1219,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1409,6 +1409,9 @@
     <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1432,12 +1435,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -9162,31 +9159,31 @@
         <v>272</v>
       </c>
       <c r="D1" s="32"/>
-      <c r="E1" s="67" t="s">
+      <c r="E1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
+      <c r="Q1" s="68"/>
+      <c r="R1" s="68"/>
+      <c r="S1" s="68"/>
+      <c r="T1" s="68"/>
+      <c r="U1" s="68"/>
+      <c r="V1" s="68"/>
+      <c r="W1" s="68"/>
+      <c r="X1" s="68"/>
+      <c r="Y1" s="68"/>
+      <c r="Z1" s="68"/>
+      <c r="AA1" s="68"/>
       <c r="AB1" s="35"/>
       <c r="AC1" s="35"/>
       <c r="AD1" s="35"/>
@@ -9472,7 +9469,9 @@
       <c r="S5" s="57">
         <v>29.9</v>
       </c>
-      <c r="T5" s="57"/>
+      <c r="T5" s="57">
+        <v>31</v>
+      </c>
       <c r="U5" s="57"/>
       <c r="V5" s="57"/>
       <c r="W5" s="57"/>
@@ -9490,7 +9489,7 @@
       <c r="AI5" s="57"/>
       <c r="AJ5" s="37">
         <f>+IF(SUM($E5:$AI5)&gt;0,LOOKUP(1000,$E5:$AI5),NA())</f>
-        <v>29.9</v>
+        <v>31</v>
       </c>
       <c r="AK5" s="21">
         <f>+MAX($E5:$AI5)</f>
@@ -9508,11 +9507,11 @@
       </c>
       <c r="AO5" s="23">
         <f>IF(COUNTIF(E5:AI5,"&gt;0")&gt;=15,AVERAGE(E5:AI5),"")</f>
-        <v>31.193333333333335</v>
+        <v>31.181250000000002</v>
       </c>
       <c r="AP5" s="23">
         <f>IF(AN5&gt;0,IFERROR(AO5-AN5,""),"")</f>
-        <v>0.99596155732510638</v>
+        <v>0.98387822399177338</v>
       </c>
     </row>
     <row r="6" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9573,7 +9572,9 @@
       <c r="S6" s="57">
         <v>29.8</v>
       </c>
-      <c r="T6" s="57"/>
+      <c r="T6" s="57">
+        <v>31.5</v>
+      </c>
       <c r="U6" s="57"/>
       <c r="V6" s="57"/>
       <c r="W6" s="57"/>
@@ -9591,7 +9592,7 @@
       <c r="AI6" s="57"/>
       <c r="AJ6" s="37">
         <f t="shared" ref="AJ6:AJ48" si="0">+IF(SUM($E6:$AI6)&gt;0,LOOKUP(1000,$E6:$AI6),NA())</f>
-        <v>29.8</v>
+        <v>31.5</v>
       </c>
       <c r="AK6" s="21">
         <f t="shared" ref="AK6:AK48" si="1">+MAX($E6:$AI6)</f>
@@ -9609,11 +9610,11 @@
       </c>
       <c r="AO6" s="23">
         <f t="shared" ref="AO6:AO15" si="3">IF(COUNTIF(E6:AI6,"&gt;0")&gt;=15,AVERAGE(E6:AI6),"")</f>
-        <v>30.533333333333328</v>
+        <v>30.593749999999996</v>
       </c>
       <c r="AP6" s="23">
         <f t="shared" ref="AP6:AP48" si="4">IF(AN6&gt;0,IFERROR(AO6-AN6,""),"")</f>
-        <v>-0.12094706368901242</v>
+        <v>-6.0530397022343863E-2</v>
       </c>
     </row>
     <row r="7" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9671,10 +9672,12 @@
       <c r="R7" s="57">
         <v>37</v>
       </c>
-      <c r="S7" s="79">
+      <c r="S7" s="67">
         <v>38.6</v>
       </c>
-      <c r="T7" s="57"/>
+      <c r="T7" s="57">
+        <v>38.299999999999997</v>
+      </c>
       <c r="U7" s="57"/>
       <c r="V7" s="57"/>
       <c r="W7" s="57"/>
@@ -9692,7 +9695,7 @@
       <c r="AI7" s="57"/>
       <c r="AJ7" s="37">
         <f t="shared" si="0"/>
-        <v>38.6</v>
+        <v>38.299999999999997</v>
       </c>
       <c r="AK7" s="21">
         <f t="shared" si="1"/>
@@ -9710,11 +9713,11 @@
       </c>
       <c r="AO7" s="23">
         <f t="shared" si="3"/>
-        <v>35.906666666666666</v>
+        <v>36.056249999999999</v>
       </c>
       <c r="AP7" s="23">
         <f t="shared" si="4"/>
-        <v>2.5406506590975937</v>
+        <v>2.690233992430926</v>
       </c>
     </row>
     <row r="8" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9775,7 +9778,9 @@
       <c r="S8" s="57">
         <v>33.799999999999997</v>
       </c>
-      <c r="T8" s="57"/>
+      <c r="T8" s="57">
+        <v>34.5</v>
+      </c>
       <c r="U8" s="57"/>
       <c r="V8" s="57"/>
       <c r="W8" s="57"/>
@@ -9793,7 +9798,7 @@
       <c r="AI8" s="57"/>
       <c r="AJ8" s="37">
         <f t="shared" si="0"/>
-        <v>33.799999999999997</v>
+        <v>34.5</v>
       </c>
       <c r="AK8" s="21">
         <f t="shared" si="1"/>
@@ -9811,11 +9816,11 @@
       </c>
       <c r="AO8" s="23">
         <f t="shared" si="3"/>
-        <v>33.326666666666668</v>
+        <v>33.400000000000006</v>
       </c>
       <c r="AP8" s="23">
         <f t="shared" si="4"/>
-        <v>1.0776236559139747</v>
+        <v>1.1509569892473124</v>
       </c>
     </row>
     <row r="9" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9876,7 +9881,9 @@
       <c r="S9" s="57">
         <v>34.700000000000003</v>
       </c>
-      <c r="T9" s="57"/>
+      <c r="T9" s="57">
+        <v>33.200000000000003</v>
+      </c>
       <c r="U9" s="57"/>
       <c r="V9" s="57"/>
       <c r="W9" s="57"/>
@@ -9894,7 +9901,7 @@
       <c r="AI9" s="57"/>
       <c r="AJ9" s="37">
         <f t="shared" si="0"/>
-        <v>34.700000000000003</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="AK9" s="21">
         <f t="shared" si="1"/>
@@ -9912,11 +9919,11 @@
       </c>
       <c r="AO9" s="23">
         <f t="shared" si="3"/>
-        <v>34.026666666666664</v>
+        <v>33.974999999999994</v>
       </c>
       <c r="AP9" s="23">
         <f t="shared" si="4"/>
-        <v>0.93542052898281725</v>
+        <v>0.88375386231614783</v>
       </c>
     </row>
     <row r="10" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9977,7 +9984,9 @@
       <c r="S10" s="57">
         <v>37</v>
       </c>
-      <c r="T10" s="57"/>
+      <c r="T10" s="57">
+        <v>35.700000000000003</v>
+      </c>
       <c r="U10" s="57"/>
       <c r="V10" s="57"/>
       <c r="W10" s="57"/>
@@ -9995,7 +10004,7 @@
       <c r="AI10" s="57"/>
       <c r="AJ10" s="37">
         <f t="shared" si="0"/>
-        <v>37</v>
+        <v>35.700000000000003</v>
       </c>
       <c r="AK10" s="21">
         <f t="shared" si="1"/>
@@ -10013,11 +10022,11 @@
       </c>
       <c r="AO10" s="23">
         <f t="shared" si="3"/>
-        <v>35.726666666666667</v>
+        <v>35.725000000000001</v>
       </c>
       <c r="AP10" s="23">
         <f t="shared" si="4"/>
-        <v>0.34642843900630993</v>
+        <v>0.34476177233964478</v>
       </c>
     </row>
     <row r="11" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10075,10 +10084,12 @@
       <c r="R11" s="57">
         <v>40.4</v>
       </c>
-      <c r="S11" s="80">
+      <c r="S11" s="57">
         <v>40.4</v>
       </c>
-      <c r="T11" s="57"/>
+      <c r="T11" s="57">
+        <v>38.799999999999997</v>
+      </c>
       <c r="U11" s="57"/>
       <c r="V11" s="57"/>
       <c r="W11" s="57"/>
@@ -10096,7 +10107,7 @@
       <c r="AI11" s="57"/>
       <c r="AJ11" s="37">
         <f t="shared" si="0"/>
-        <v>40.4</v>
+        <v>38.799999999999997</v>
       </c>
       <c r="AK11" s="21">
         <f t="shared" si="1"/>
@@ -10114,11 +10125,11 @@
       </c>
       <c r="AO11" s="23">
         <f t="shared" si="3"/>
-        <v>38.239999999999995</v>
+        <v>38.274999999999991</v>
       </c>
       <c r="AP11" s="23">
         <f t="shared" si="4"/>
-        <v>2.7027159071513935</v>
+        <v>2.7377159071513901</v>
       </c>
     </row>
     <row r="12" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10179,7 +10190,9 @@
       <c r="S12" s="57">
         <v>36.200000000000003</v>
       </c>
-      <c r="T12" s="57"/>
+      <c r="T12" s="57">
+        <v>36.4</v>
+      </c>
       <c r="U12" s="57"/>
       <c r="V12" s="57"/>
       <c r="W12" s="57"/>
@@ -10197,7 +10210,7 @@
       <c r="AI12" s="57"/>
       <c r="AJ12" s="37">
         <f t="shared" si="0"/>
-        <v>36.200000000000003</v>
+        <v>36.4</v>
       </c>
       <c r="AK12" s="21">
         <f t="shared" si="1"/>
@@ -10215,11 +10228,11 @@
       </c>
       <c r="AO12" s="23">
         <f t="shared" si="3"/>
-        <v>34.840000000000003</v>
+        <v>34.9375</v>
       </c>
       <c r="AP12" s="23">
         <f t="shared" si="4"/>
-        <v>2.6513758538262664</v>
+        <v>2.748875853826263</v>
       </c>
     </row>
     <row r="13" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10280,7 +10293,9 @@
       <c r="S13" s="57">
         <v>37.6</v>
       </c>
-      <c r="T13" s="57"/>
+      <c r="T13" s="57">
+        <v>37.799999999999997</v>
+      </c>
       <c r="U13" s="57"/>
       <c r="V13" s="57"/>
       <c r="W13" s="57"/>
@@ -10298,7 +10313,7 @@
       <c r="AI13" s="57"/>
       <c r="AJ13" s="37">
         <f t="shared" si="0"/>
-        <v>37.6</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="AK13" s="21">
         <f t="shared" si="1"/>
@@ -10316,11 +10331,11 @@
       </c>
       <c r="AO13" s="23">
         <f t="shared" si="3"/>
-        <v>36.04</v>
+        <v>36.15</v>
       </c>
       <c r="AP13" s="23">
         <f t="shared" si="4"/>
-        <v>2.6582078853046625</v>
+        <v>2.7682078853046619</v>
       </c>
     </row>
     <row r="14" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10381,7 +10396,9 @@
       <c r="S14" s="57">
         <v>37.1</v>
       </c>
-      <c r="T14" s="57"/>
+      <c r="T14" s="57">
+        <v>37.5</v>
+      </c>
       <c r="U14" s="57"/>
       <c r="V14" s="57"/>
       <c r="W14" s="57"/>
@@ -10399,29 +10416,29 @@
       <c r="AI14" s="57"/>
       <c r="AJ14" s="37">
         <f t="shared" si="0"/>
-        <v>37.1</v>
+        <v>37.5</v>
       </c>
       <c r="AK14" s="21">
         <f t="shared" si="1"/>
-        <v>37.1</v>
+        <v>37.5</v>
       </c>
       <c r="AL14" s="22">
         <v>38.4</v>
       </c>
       <c r="AM14" s="23">
         <f t="shared" si="2"/>
-        <v>-1.2999999999999972</v>
+        <v>-0.89999999999999858</v>
       </c>
       <c r="AN14" s="23">
         <v>33.224936599214232</v>
       </c>
       <c r="AO14" s="23">
         <f t="shared" si="3"/>
-        <v>34.986666666666665</v>
+        <v>35.143749999999997</v>
       </c>
       <c r="AP14" s="23">
         <f t="shared" si="4"/>
-        <v>1.761730067452433</v>
+        <v>1.9188134007857656</v>
       </c>
     </row>
     <row r="15" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10482,7 +10499,9 @@
       <c r="S15" s="57">
         <v>33.1</v>
       </c>
-      <c r="T15" s="57"/>
+      <c r="T15" s="57">
+        <v>33.5</v>
+      </c>
       <c r="U15" s="57"/>
       <c r="V15" s="57"/>
       <c r="W15" s="57"/>
@@ -10500,29 +10519,29 @@
       <c r="AI15" s="57"/>
       <c r="AJ15" s="37">
         <f t="shared" si="0"/>
-        <v>33.1</v>
+        <v>33.5</v>
       </c>
       <c r="AK15" s="21">
         <f t="shared" si="1"/>
-        <v>33.4</v>
+        <v>33.5</v>
       </c>
       <c r="AL15" s="22">
         <v>36</v>
       </c>
       <c r="AM15" s="23">
         <f t="shared" si="2"/>
-        <v>-2.6000000000000014</v>
+        <v>-2.5</v>
       </c>
       <c r="AN15" s="23">
         <v>31.73533745607995</v>
       </c>
       <c r="AO15" s="23">
         <f t="shared" si="3"/>
-        <v>31.686666666666667</v>
+        <v>31.8</v>
       </c>
       <c r="AP15" s="23">
         <f t="shared" si="4"/>
-        <v>-4.8670789413282733E-2</v>
+        <v>6.4662543920050553E-2</v>
       </c>
     </row>
     <row r="16" spans="1:46" s="2" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -10632,7 +10651,9 @@
       <c r="S17" s="57">
         <v>35.6</v>
       </c>
-      <c r="T17" s="57"/>
+      <c r="T17" s="57">
+        <v>37.200000000000003</v>
+      </c>
       <c r="U17" s="57"/>
       <c r="V17" s="57"/>
       <c r="W17" s="57"/>
@@ -10650,29 +10671,29 @@
       <c r="AI17" s="57"/>
       <c r="AJ17" s="37">
         <f t="shared" si="0"/>
-        <v>35.6</v>
+        <v>37.200000000000003</v>
       </c>
       <c r="AK17" s="21">
         <f t="shared" si="1"/>
-        <v>36.299999999999997</v>
+        <v>37.200000000000003</v>
       </c>
       <c r="AL17" s="22">
         <v>37.6</v>
       </c>
       <c r="AM17" s="23">
         <f t="shared" si="2"/>
-        <v>-1.3000000000000043</v>
+        <v>-0.39999999999999858</v>
       </c>
       <c r="AN17" s="23">
         <v>32.673982202447156</v>
       </c>
       <c r="AO17" s="23">
         <f>IF(COUNTIF(E17:AI17,"&gt;0")&gt;=15,AVERAGE(E17:AI17),"")</f>
-        <v>34.273333333333326</v>
+        <v>34.456249999999997</v>
       </c>
       <c r="AP17" s="23">
         <f>IF(AN17&gt;0,IFERROR(AO17-AN17,""),"")</f>
-        <v>1.5993511308861699</v>
+        <v>1.7822677975528407</v>
       </c>
     </row>
     <row r="18" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10703,7 +10724,7 @@
       <c r="I18" s="57">
         <v>29.2</v>
       </c>
-      <c r="J18" s="79">
+      <c r="J18" s="67">
         <v>30.4</v>
       </c>
       <c r="K18" s="57">
@@ -10733,7 +10754,9 @@
       <c r="S18" s="57">
         <v>30.1</v>
       </c>
-      <c r="T18" s="57"/>
+      <c r="T18" s="57">
+        <v>30.3</v>
+      </c>
       <c r="U18" s="57"/>
       <c r="V18" s="57"/>
       <c r="W18" s="57"/>
@@ -10751,7 +10774,7 @@
       <c r="AI18" s="57"/>
       <c r="AJ18" s="37">
         <f t="shared" si="0"/>
-        <v>30.1</v>
+        <v>30.3</v>
       </c>
       <c r="AK18" s="21">
         <f t="shared" si="1"/>
@@ -10769,11 +10792,11 @@
       </c>
       <c r="AO18" s="23">
         <f t="shared" ref="AO18:AO33" si="5">IF(COUNTIF(E18:AI18,"&gt;0")&gt;=15,AVERAGE(E18:AI18),"")</f>
-        <v>27.880000000000003</v>
+        <v>28.031250000000004</v>
       </c>
       <c r="AP18" s="23">
         <f t="shared" si="4"/>
-        <v>1.8201291460431328</v>
+        <v>1.9713791460431338</v>
       </c>
     </row>
     <row r="19" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10834,7 +10857,9 @@
       <c r="S19" s="57">
         <v>35.700000000000003</v>
       </c>
-      <c r="T19" s="57"/>
+      <c r="T19" s="57">
+        <v>33.700000000000003</v>
+      </c>
       <c r="U19" s="57"/>
       <c r="V19" s="57"/>
       <c r="W19" s="57"/>
@@ -10852,7 +10877,7 @@
       <c r="AI19" s="57"/>
       <c r="AJ19" s="37">
         <f t="shared" si="0"/>
-        <v>35.700000000000003</v>
+        <v>33.700000000000003</v>
       </c>
       <c r="AK19" s="21">
         <f t="shared" si="1"/>
@@ -10870,11 +10895,11 @@
       </c>
       <c r="AO19" s="23">
         <f t="shared" si="5"/>
-        <v>33.813333333333325</v>
+        <v>33.806249999999999</v>
       </c>
       <c r="AP19" s="23">
         <f t="shared" si="4"/>
-        <v>0.5623709306636826</v>
+        <v>0.55528759733035571</v>
       </c>
     </row>
     <row r="20" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10908,7 +10933,7 @@
       <c r="J20" s="57">
         <v>32</v>
       </c>
-      <c r="K20" s="79">
+      <c r="K20" s="67">
         <v>34.5</v>
       </c>
       <c r="L20" s="57">
@@ -10935,7 +10960,9 @@
       <c r="S20" s="57">
         <v>31.1</v>
       </c>
-      <c r="T20" s="57"/>
+      <c r="T20" s="57">
+        <v>31.1</v>
+      </c>
       <c r="U20" s="57"/>
       <c r="V20" s="57"/>
       <c r="W20" s="57"/>
@@ -10971,11 +10998,11 @@
       </c>
       <c r="AO20" s="23">
         <f t="shared" si="5"/>
-        <v>30.54666666666667</v>
+        <v>30.581250000000004</v>
       </c>
       <c r="AP20" s="23">
         <f t="shared" si="4"/>
-        <v>1.9058620689655221</v>
+        <v>1.940445402298856</v>
       </c>
     </row>
     <row r="21" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11009,7 +11036,7 @@
       <c r="J21" s="57">
         <v>25.4</v>
       </c>
-      <c r="K21" s="79">
+      <c r="K21" s="67">
         <v>26.1</v>
       </c>
       <c r="L21" s="57">
@@ -11036,7 +11063,9 @@
       <c r="S21" s="57">
         <v>24.4</v>
       </c>
-      <c r="T21" s="57"/>
+      <c r="T21" s="57">
+        <v>24.6</v>
+      </c>
       <c r="U21" s="57"/>
       <c r="V21" s="57"/>
       <c r="W21" s="57"/>
@@ -11054,7 +11083,7 @@
       <c r="AI21" s="57"/>
       <c r="AJ21" s="37">
         <f t="shared" si="0"/>
-        <v>24.4</v>
+        <v>24.6</v>
       </c>
       <c r="AK21" s="21">
         <f t="shared" si="1"/>
@@ -11072,11 +11101,11 @@
       </c>
       <c r="AO21" s="23">
         <f t="shared" si="5"/>
-        <v>24.386666666666663</v>
+        <v>24.4</v>
       </c>
       <c r="AP21" s="23">
         <f t="shared" si="4"/>
-        <v>1.7771635150166922</v>
+        <v>1.7904968483500276</v>
       </c>
     </row>
     <row r="22" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11205,7 +11234,9 @@
       <c r="S23" s="57">
         <v>29.5</v>
       </c>
-      <c r="T23" s="57"/>
+      <c r="T23" s="57">
+        <v>30.8</v>
+      </c>
       <c r="U23" s="57"/>
       <c r="V23" s="57"/>
       <c r="W23" s="57"/>
@@ -11223,7 +11254,7 @@
       <c r="AI23" s="57"/>
       <c r="AJ23" s="37">
         <f t="shared" si="0"/>
-        <v>29.5</v>
+        <v>30.8</v>
       </c>
       <c r="AK23" s="21">
         <f t="shared" si="1"/>
@@ -11241,11 +11272,11 @@
       </c>
       <c r="AO23" s="23">
         <f t="shared" si="5"/>
-        <v>28.793333333333337</v>
+        <v>28.918750000000003</v>
       </c>
       <c r="AP23" s="23">
         <f t="shared" si="4"/>
-        <v>1.924946236559137</v>
+        <v>2.0503629032258033</v>
       </c>
     </row>
     <row r="24" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11303,10 +11334,12 @@
       <c r="R24" s="57">
         <v>31.4</v>
       </c>
-      <c r="S24" s="80">
+      <c r="S24" s="57">
         <v>31.4</v>
       </c>
-      <c r="T24" s="57"/>
+      <c r="T24" s="57">
+        <v>32.799999999999997</v>
+      </c>
       <c r="U24" s="57"/>
       <c r="V24" s="57"/>
       <c r="W24" s="57"/>
@@ -11324,7 +11357,7 @@
       <c r="AI24" s="57"/>
       <c r="AJ24" s="37">
         <f t="shared" si="0"/>
-        <v>31.4</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="AK24" s="21">
         <f t="shared" si="1"/>
@@ -11342,11 +11375,11 @@
       </c>
       <c r="AO24" s="23">
         <f t="shared" si="5"/>
-        <v>29.993333333333332</v>
+        <v>30.168749999999999</v>
       </c>
       <c r="AP24" s="23">
         <f t="shared" si="4"/>
-        <v>1.7415092165898507</v>
+        <v>1.9169258832565177</v>
       </c>
     </row>
     <row r="25" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11407,7 +11440,9 @@
       <c r="S25" s="57">
         <v>34.6</v>
       </c>
-      <c r="T25" s="57"/>
+      <c r="T25" s="57">
+        <v>33.299999999999997</v>
+      </c>
       <c r="U25" s="57"/>
       <c r="V25" s="57"/>
       <c r="W25" s="57"/>
@@ -11425,7 +11460,7 @@
       <c r="AI25" s="57"/>
       <c r="AJ25" s="37">
         <f t="shared" si="0"/>
-        <v>34.6</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="AK25" s="21">
         <f t="shared" si="1"/>
@@ -11443,11 +11478,11 @@
       </c>
       <c r="AO25" s="23">
         <f t="shared" si="5"/>
-        <v>32.260000000000005</v>
+        <v>32.325000000000003</v>
       </c>
       <c r="AP25" s="23">
         <f t="shared" si="4"/>
-        <v>1.884134606778936</v>
+        <v>1.9491346067789337</v>
       </c>
     </row>
     <row r="26" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11508,7 +11543,9 @@
       <c r="S26" s="57">
         <v>19.5</v>
       </c>
-      <c r="T26" s="57"/>
+      <c r="T26" s="57">
+        <v>21.6</v>
+      </c>
       <c r="U26" s="57"/>
       <c r="V26" s="57"/>
       <c r="W26" s="57"/>
@@ -11526,29 +11563,29 @@
       <c r="AI26" s="57"/>
       <c r="AJ26" s="37">
         <f t="shared" si="0"/>
-        <v>19.5</v>
+        <v>21.6</v>
       </c>
       <c r="AK26" s="21">
         <f t="shared" si="1"/>
-        <v>21</v>
+        <v>21.6</v>
       </c>
       <c r="AL26" s="22">
         <v>22.4</v>
       </c>
       <c r="AM26" s="23">
         <f t="shared" si="2"/>
-        <v>-1.3999999999999986</v>
+        <v>-0.79999999999999716</v>
       </c>
       <c r="AN26" s="23">
         <v>18.542871607443359</v>
       </c>
       <c r="AO26" s="23">
         <f t="shared" si="5"/>
-        <v>19.453333333333333</v>
+        <v>19.587500000000002</v>
       </c>
       <c r="AP26" s="23">
         <f t="shared" si="4"/>
-        <v>0.91046172588997365</v>
+        <v>1.0446283925566426</v>
       </c>
     </row>
     <row r="27" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11606,10 +11643,12 @@
       <c r="R27" s="57">
         <v>20.399999999999999</v>
       </c>
-      <c r="S27" s="79">
+      <c r="S27" s="67">
         <v>21.6</v>
       </c>
-      <c r="T27" s="57"/>
+      <c r="T27" s="57">
+        <v>19.399999999999999</v>
+      </c>
       <c r="U27" s="57"/>
       <c r="V27" s="57"/>
       <c r="W27" s="57"/>
@@ -11627,7 +11666,7 @@
       <c r="AI27" s="57"/>
       <c r="AJ27" s="37">
         <f t="shared" si="0"/>
-        <v>21.6</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="AK27" s="21">
         <f t="shared" si="1"/>
@@ -11645,11 +11684,11 @@
       </c>
       <c r="AO27" s="23">
         <f t="shared" si="5"/>
-        <v>18.059999999999999</v>
+        <v>18.143749999999997</v>
       </c>
       <c r="AP27" s="23">
         <f t="shared" si="4"/>
-        <v>1.3779494558916099</v>
+        <v>1.4616994558916083</v>
       </c>
     </row>
     <row r="28" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11683,7 +11722,7 @@
       <c r="J28" s="57">
         <v>33.9</v>
       </c>
-      <c r="K28" s="79">
+      <c r="K28" s="67">
         <v>35.5</v>
       </c>
       <c r="L28" s="57">
@@ -11710,7 +11749,9 @@
       <c r="S28" s="57">
         <v>34.6</v>
       </c>
-      <c r="T28" s="57"/>
+      <c r="T28" s="57">
+        <v>32.299999999999997</v>
+      </c>
       <c r="U28" s="57"/>
       <c r="V28" s="57"/>
       <c r="W28" s="57"/>
@@ -11728,7 +11769,7 @@
       <c r="AI28" s="57"/>
       <c r="AJ28" s="37">
         <f t="shared" si="0"/>
-        <v>34.6</v>
+        <v>32.299999999999997</v>
       </c>
       <c r="AK28" s="21">
         <f t="shared" si="1"/>
@@ -11746,11 +11787,11 @@
       </c>
       <c r="AO28" s="23">
         <f t="shared" si="5"/>
-        <v>32.266666666666673</v>
+        <v>32.268750000000004</v>
       </c>
       <c r="AP28" s="23">
         <f t="shared" si="4"/>
-        <v>1.7382140650105136</v>
+        <v>1.740297398343845</v>
       </c>
     </row>
     <row r="29" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11877,7 +11918,9 @@
       <c r="S30" s="57">
         <v>36.200000000000003</v>
       </c>
-      <c r="T30" s="57"/>
+      <c r="T30" s="57">
+        <v>35.299999999999997</v>
+      </c>
       <c r="U30" s="57"/>
       <c r="V30" s="57"/>
       <c r="W30" s="57"/>
@@ -11895,7 +11938,7 @@
       <c r="AI30" s="57"/>
       <c r="AJ30" s="37">
         <f t="shared" si="0"/>
-        <v>36.200000000000003</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="AK30" s="21">
         <f t="shared" si="1"/>
@@ -11913,11 +11956,11 @@
       </c>
       <c r="AO30" s="23">
         <f t="shared" si="5"/>
-        <v>34.600000000000009</v>
+        <v>34.643750000000004</v>
       </c>
       <c r="AP30" s="23">
         <f t="shared" si="4"/>
-        <v>0.85774910394265902</v>
+        <v>0.90149910394265476</v>
       </c>
     </row>
     <row r="31" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11978,7 +12021,9 @@
       <c r="S31" s="57">
         <v>28.6</v>
       </c>
-      <c r="T31" s="57"/>
+      <c r="T31" s="57">
+        <v>29.4</v>
+      </c>
       <c r="U31" s="57"/>
       <c r="V31" s="57"/>
       <c r="W31" s="57"/>
@@ -11996,29 +12041,29 @@
       <c r="AI31" s="57"/>
       <c r="AJ31" s="37">
         <f t="shared" si="0"/>
-        <v>28.6</v>
+        <v>29.4</v>
       </c>
       <c r="AK31" s="21">
         <f t="shared" si="1"/>
-        <v>29.2</v>
+        <v>29.4</v>
       </c>
       <c r="AL31" s="22">
         <v>30.2</v>
       </c>
       <c r="AM31" s="23">
         <f t="shared" si="2"/>
-        <v>-1</v>
+        <v>-0.80000000000000071</v>
       </c>
       <c r="AN31" s="23">
         <v>25.387424837120619</v>
       </c>
       <c r="AO31" s="23">
         <f t="shared" si="5"/>
-        <v>27.700000000000003</v>
+        <v>27.806250000000002</v>
       </c>
       <c r="AP31" s="23">
         <f t="shared" si="4"/>
-        <v>2.3125751628793836</v>
+        <v>2.4188251628793829</v>
       </c>
     </row>
     <row r="32" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12079,7 +12124,9 @@
       <c r="S32" s="57">
         <v>18.2</v>
       </c>
-      <c r="T32" s="57"/>
+      <c r="T32" s="57">
+        <v>18</v>
+      </c>
       <c r="U32" s="57"/>
       <c r="V32" s="57"/>
       <c r="W32" s="57"/>
@@ -12097,7 +12144,7 @@
       <c r="AI32" s="57"/>
       <c r="AJ32" s="37">
         <f t="shared" si="0"/>
-        <v>18.2</v>
+        <v>18</v>
       </c>
       <c r="AK32" s="21">
         <f t="shared" si="1"/>
@@ -12115,11 +12162,11 @@
       </c>
       <c r="AO32" s="23">
         <f t="shared" si="5"/>
-        <v>17.853333333333335</v>
+        <v>17.862500000000001</v>
       </c>
       <c r="AP32" s="23">
         <f t="shared" si="4"/>
-        <v>1.5237955600720845</v>
+        <v>1.5329622267387499</v>
       </c>
     </row>
     <row r="33" spans="1:47" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12180,7 +12227,9 @@
       <c r="S33" s="57">
         <v>16</v>
       </c>
-      <c r="T33" s="57"/>
+      <c r="T33" s="57">
+        <v>16.399999999999999</v>
+      </c>
       <c r="U33" s="57"/>
       <c r="V33" s="57"/>
       <c r="W33" s="57"/>
@@ -12198,7 +12247,7 @@
       <c r="AI33" s="57"/>
       <c r="AJ33" s="37">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="AK33" s="21">
         <f t="shared" si="1"/>
@@ -12216,11 +12265,11 @@
       </c>
       <c r="AO33" s="23">
         <f t="shared" si="5"/>
-        <v>15.62</v>
+        <v>15.668749999999999</v>
       </c>
       <c r="AP33" s="23">
         <f t="shared" si="4"/>
-        <v>0.87538746755654984</v>
+        <v>0.92413746755654991</v>
       </c>
       <c r="AT33" s="15"/>
     </row>
@@ -12333,7 +12382,9 @@
       <c r="S35" s="57">
         <v>30.8</v>
       </c>
-      <c r="T35" s="57"/>
+      <c r="T35" s="57">
+        <v>34.6</v>
+      </c>
       <c r="U35" s="57"/>
       <c r="V35" s="57"/>
       <c r="W35" s="57"/>
@@ -12351,7 +12402,7 @@
       <c r="AI35" s="57"/>
       <c r="AJ35" s="37">
         <f t="shared" si="0"/>
-        <v>30.8</v>
+        <v>34.6</v>
       </c>
       <c r="AK35" s="21">
         <f t="shared" si="1"/>
@@ -12369,11 +12420,11 @@
       </c>
       <c r="AO35" s="23">
         <f>IF(COUNTIF(E35:AI35,"&gt;0")&gt;=15,AVERAGE(E35:AI35),"")</f>
-        <v>31.999999999999996</v>
+        <v>32.162499999999994</v>
       </c>
       <c r="AP35" s="23">
         <f t="shared" si="4"/>
-        <v>0.92730414746543488</v>
+        <v>1.0898041474654327</v>
       </c>
       <c r="AT35" s="15"/>
     </row>
@@ -12555,7 +12606,9 @@
       <c r="S38" s="57">
         <v>32.4</v>
       </c>
-      <c r="T38" s="57"/>
+      <c r="T38" s="57">
+        <v>32.200000000000003</v>
+      </c>
       <c r="U38" s="57"/>
       <c r="V38" s="57"/>
       <c r="W38" s="57"/>
@@ -12573,7 +12626,7 @@
       <c r="AI38" s="57"/>
       <c r="AJ38" s="37">
         <f t="shared" si="0"/>
-        <v>32.4</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AK38" s="21">
         <f t="shared" si="1"/>
@@ -12591,11 +12644,11 @@
       </c>
       <c r="AO38" s="23">
         <f>IF(COUNTIF(E38:AI38,"&gt;0")&gt;=15,AVERAGE(E38:AI38),"")</f>
-        <v>29.766666666666662</v>
+        <v>29.918749999999996</v>
       </c>
       <c r="AP38" s="23">
         <f t="shared" si="4"/>
-        <v>-0.26235955672591871</v>
+        <v>-0.11027622339258514</v>
       </c>
       <c r="AT38" s="15"/>
     </row>
@@ -12657,7 +12710,9 @@
       <c r="S39" s="57">
         <v>33.6</v>
       </c>
-      <c r="T39" s="57"/>
+      <c r="T39" s="57">
+        <v>33.4</v>
+      </c>
       <c r="U39" s="57"/>
       <c r="V39" s="57"/>
       <c r="W39" s="57"/>
@@ -12675,7 +12730,7 @@
       <c r="AI39" s="57"/>
       <c r="AJ39" s="37">
         <f t="shared" si="0"/>
-        <v>33.6</v>
+        <v>33.4</v>
       </c>
       <c r="AK39" s="21">
         <f t="shared" si="1"/>
@@ -12693,11 +12748,11 @@
       </c>
       <c r="AO39" s="23">
         <f t="shared" ref="AO39:AO48" si="7">IF(COUNTIF(E39:AI39,"&gt;0")&gt;=15,AVERAGE(E39:AI39),"")</f>
-        <v>31.066666666666666</v>
+        <v>31.212499999999999</v>
       </c>
       <c r="AP39" s="23">
         <f t="shared" si="4"/>
-        <v>0.22353355580274581</v>
+        <v>0.36936688913607796</v>
       </c>
       <c r="AT39" s="15"/>
     </row>
@@ -12759,7 +12814,9 @@
       <c r="S40" s="57">
         <v>30.6</v>
       </c>
-      <c r="T40" s="57"/>
+      <c r="T40" s="57">
+        <v>30.2</v>
+      </c>
       <c r="U40" s="57"/>
       <c r="V40" s="57"/>
       <c r="W40" s="57"/>
@@ -12777,7 +12834,7 @@
       <c r="AI40" s="57"/>
       <c r="AJ40" s="37">
         <f t="shared" si="0"/>
-        <v>30.6</v>
+        <v>30.2</v>
       </c>
       <c r="AK40" s="21">
         <f t="shared" si="1"/>
@@ -12795,11 +12852,11 @@
       </c>
       <c r="AO40" s="23">
         <f t="shared" si="7"/>
-        <v>29.24666666666667</v>
+        <v>29.306250000000002</v>
       </c>
       <c r="AP40" s="23">
         <f t="shared" si="4"/>
-        <v>0.29911827956988901</v>
+        <v>0.35870161290322145</v>
       </c>
       <c r="AT40" s="15"/>
     </row>
@@ -12861,7 +12918,9 @@
       <c r="S41" s="57">
         <v>33.4</v>
       </c>
-      <c r="T41" s="57"/>
+      <c r="T41" s="57">
+        <v>33.200000000000003</v>
+      </c>
       <c r="U41" s="57"/>
       <c r="V41" s="57"/>
       <c r="W41" s="57"/>
@@ -12879,7 +12938,7 @@
       <c r="AI41" s="57"/>
       <c r="AJ41" s="37">
         <f t="shared" si="0"/>
-        <v>33.4</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="AK41" s="21">
         <f t="shared" si="1"/>
@@ -12897,11 +12956,11 @@
       </c>
       <c r="AO41" s="23">
         <f t="shared" si="7"/>
-        <v>30.106666666666669</v>
+        <v>30.3</v>
       </c>
       <c r="AP41" s="23">
         <f t="shared" si="4"/>
-        <v>0.74035842293907805</v>
+        <v>0.93369175627240963</v>
       </c>
       <c r="AT41" s="15"/>
     </row>
@@ -13024,7 +13083,9 @@
       <c r="S43" s="57">
         <v>31.6</v>
       </c>
-      <c r="T43" s="57"/>
+      <c r="T43" s="57">
+        <v>33.200000000000003</v>
+      </c>
       <c r="U43" s="57"/>
       <c r="V43" s="57"/>
       <c r="W43" s="57"/>
@@ -13042,18 +13103,18 @@
       <c r="AI43" s="57"/>
       <c r="AJ43" s="37">
         <f t="shared" si="0"/>
-        <v>31.6</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="AK43" s="21">
         <f t="shared" si="1"/>
-        <v>32</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="AL43" s="22">
         <v>34.200000000000003</v>
       </c>
       <c r="AM43" s="23">
         <f t="shared" si="2"/>
-        <v>-2.2000000000000028</v>
+        <v>-1</v>
       </c>
       <c r="AN43" s="23">
         <v>30.061061827956991</v>
@@ -13124,7 +13185,9 @@
       <c r="S44" s="29">
         <v>31.2</v>
       </c>
-      <c r="T44" s="29"/>
+      <c r="T44" s="29">
+        <v>31.2</v>
+      </c>
       <c r="U44" s="29"/>
       <c r="V44" s="29"/>
       <c r="W44" s="29"/>
@@ -13158,13 +13221,13 @@
       <c r="AN44" s="23">
         <v>29.043187205360461</v>
       </c>
-      <c r="AO44" s="23" t="str">
+      <c r="AO44" s="23">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="AP44" s="23" t="str">
+        <v>31.213333333333331</v>
+      </c>
+      <c r="AP44" s="23">
         <f t="shared" si="4"/>
-        <v/>
+        <v>2.1701461279728704</v>
       </c>
       <c r="AT44" s="15"/>
     </row>
@@ -13226,7 +13289,9 @@
       <c r="S45" s="57">
         <v>31.6</v>
       </c>
-      <c r="T45" s="57"/>
+      <c r="T45" s="57">
+        <v>32.799999999999997</v>
+      </c>
       <c r="U45" s="57"/>
       <c r="V45" s="57"/>
       <c r="W45" s="57"/>
@@ -13244,7 +13309,7 @@
       <c r="AI45" s="57"/>
       <c r="AJ45" s="37">
         <f t="shared" si="0"/>
-        <v>31.6</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="AK45" s="21">
         <f t="shared" si="1"/>
@@ -13262,11 +13327,11 @@
       </c>
       <c r="AO45" s="23">
         <f t="shared" si="7"/>
-        <v>30.13333333333334</v>
+        <v>30.300000000000008</v>
       </c>
       <c r="AP45" s="23">
         <f t="shared" si="4"/>
-        <v>0.58751694045450975</v>
+        <v>0.7541836071211776</v>
       </c>
       <c r="AT45" s="15"/>
     </row>
@@ -13467,7 +13532,9 @@
       <c r="S48" s="57">
         <v>29.2</v>
       </c>
-      <c r="T48" s="57"/>
+      <c r="T48" s="57">
+        <v>31.9</v>
+      </c>
       <c r="U48" s="57"/>
       <c r="V48" s="57"/>
       <c r="W48" s="57"/>
@@ -13485,7 +13552,7 @@
       <c r="AI48" s="57"/>
       <c r="AJ48" s="37">
         <f t="shared" si="0"/>
-        <v>29.2</v>
+        <v>31.9</v>
       </c>
       <c r="AK48" s="21">
         <f t="shared" si="1"/>
@@ -13503,11 +13570,11 @@
       </c>
       <c r="AO48" s="23">
         <f t="shared" si="7"/>
-        <v>29.806666666666668</v>
+        <v>29.9375</v>
       </c>
       <c r="AP48" s="23">
         <f t="shared" si="4"/>
-        <v>-0.53586618876941117</v>
+        <v>-0.40503285543607959</v>
       </c>
     </row>
     <row r="49" spans="5:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -19849,66 +19916,66 @@
       <c r="E1" s="52"/>
       <c r="F1" s="52"/>
       <c r="G1" s="52"/>
-      <c r="H1" s="71" t="s">
+      <c r="H1" s="72" t="s">
         <v>123</v>
       </c>
-      <c r="I1" s="72"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="68" t="s">
+      <c r="I1" s="73"/>
+      <c r="J1" s="74"/>
+      <c r="K1" s="69" t="s">
         <v>124</v>
       </c>
-      <c r="L1" s="69"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="71" t="s">
+      <c r="L1" s="70"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="72" t="s">
         <v>125</v>
       </c>
-      <c r="O1" s="72"/>
-      <c r="P1" s="73"/>
-      <c r="Q1" s="68" t="s">
+      <c r="O1" s="73"/>
+      <c r="P1" s="74"/>
+      <c r="Q1" s="69" t="s">
         <v>126</v>
       </c>
-      <c r="R1" s="69"/>
-      <c r="S1" s="70"/>
-      <c r="T1" s="71" t="s">
+      <c r="R1" s="70"/>
+      <c r="S1" s="71"/>
+      <c r="T1" s="72" t="s">
         <v>127</v>
       </c>
-      <c r="U1" s="72"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="68" t="s">
+      <c r="U1" s="73"/>
+      <c r="V1" s="74"/>
+      <c r="W1" s="69" t="s">
         <v>128</v>
       </c>
-      <c r="X1" s="69"/>
-      <c r="Y1" s="70"/>
-      <c r="Z1" s="71" t="s">
+      <c r="X1" s="70"/>
+      <c r="Y1" s="71"/>
+      <c r="Z1" s="72" t="s">
         <v>129</v>
       </c>
-      <c r="AA1" s="72"/>
-      <c r="AB1" s="73"/>
-      <c r="AC1" s="68" t="s">
+      <c r="AA1" s="73"/>
+      <c r="AB1" s="74"/>
+      <c r="AC1" s="69" t="s">
         <v>130</v>
       </c>
-      <c r="AD1" s="69"/>
-      <c r="AE1" s="70"/>
-      <c r="AF1" s="71" t="s">
+      <c r="AD1" s="70"/>
+      <c r="AE1" s="71"/>
+      <c r="AF1" s="72" t="s">
         <v>131</v>
       </c>
-      <c r="AG1" s="72"/>
-      <c r="AH1" s="73"/>
-      <c r="AI1" s="68" t="s">
+      <c r="AG1" s="73"/>
+      <c r="AH1" s="74"/>
+      <c r="AI1" s="69" t="s">
         <v>132</v>
       </c>
-      <c r="AJ1" s="69"/>
-      <c r="AK1" s="70"/>
-      <c r="AL1" s="71" t="s">
+      <c r="AJ1" s="70"/>
+      <c r="AK1" s="71"/>
+      <c r="AL1" s="72" t="s">
         <v>133</v>
       </c>
-      <c r="AM1" s="72"/>
-      <c r="AN1" s="73"/>
-      <c r="AO1" s="68" t="s">
+      <c r="AM1" s="73"/>
+      <c r="AN1" s="74"/>
+      <c r="AO1" s="69" t="s">
         <v>134</v>
       </c>
-      <c r="AP1" s="69"/>
-      <c r="AQ1" s="70"/>
+      <c r="AP1" s="70"/>
+      <c r="AQ1" s="71"/>
     </row>
     <row r="2" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A2" s="54" t="s">
@@ -25345,68 +25412,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="78" t="s">
+      <c r="B1" s="79" t="s">
         <v>93</v>
       </c>
-      <c r="C1" s="67" t="s">
+      <c r="C1" s="68" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="74" t="s">
+      <c r="D1" s="75" t="s">
         <v>95</v>
       </c>
-      <c r="E1" s="74" t="s">
+      <c r="E1" s="75" t="s">
         <v>96</v>
       </c>
-      <c r="F1" s="74" t="s">
+      <c r="F1" s="75" t="s">
         <v>97</v>
       </c>
-      <c r="G1" s="74" t="s">
+      <c r="G1" s="75" t="s">
         <v>98</v>
       </c>
-      <c r="H1" s="74" t="s">
+      <c r="H1" s="75" t="s">
         <v>99</v>
       </c>
-      <c r="I1" s="74" t="s">
+      <c r="I1" s="75" t="s">
         <v>100</v>
       </c>
-      <c r="J1" s="74" t="s">
+      <c r="J1" s="75" t="s">
         <v>101</v>
       </c>
-      <c r="K1" s="74" t="s">
+      <c r="K1" s="75" t="s">
         <v>102</v>
       </c>
-      <c r="L1" s="74" t="s">
+      <c r="L1" s="75" t="s">
         <v>103</v>
       </c>
-      <c r="M1" s="74" t="s">
+      <c r="M1" s="75" t="s">
         <v>104</v>
       </c>
-      <c r="N1" s="74" t="s">
+      <c r="N1" s="75" t="s">
         <v>105</v>
       </c>
-      <c r="O1" s="74" t="s">
+      <c r="O1" s="75" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="77"/>
-      <c r="B2" s="75"/>
-      <c r="C2" s="75"/>
-      <c r="D2" s="75"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="75"/>
-      <c r="G2" s="75"/>
-      <c r="H2" s="75"/>
-      <c r="I2" s="75"/>
-      <c r="J2" s="75"/>
-      <c r="K2" s="75"/>
-      <c r="L2" s="75"/>
-      <c r="M2" s="75"/>
-      <c r="N2" s="75"/>
-      <c r="O2" s="75"/>
+      <c r="A2" s="78"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
+      <c r="G2" s="76"/>
+      <c r="H2" s="76"/>
+      <c r="I2" s="76"/>
+      <c r="J2" s="76"/>
+      <c r="K2" s="76"/>
+      <c r="L2" s="76"/>
+      <c r="M2" s="76"/>
+      <c r="N2" s="76"/>
+      <c r="O2" s="76"/>
     </row>
     <row r="3" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
@@ -26406,12 +26473,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
     <mergeCell ref="O1:O2"/>
@@ -26421,6 +26482,12 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="L1:L2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:O13 D15:O31 D33:O34 D36:O46">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>